<commit_message>
Ajoute coachs sous forme de liste update testunit
</commit_message>
<xml_diff>
--- a/backend/template.xlsx
+++ b/backend/template.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\c.lhermitte\Documents\Workspace\aslb\basket\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE48126A-D2C9-4FA0-A9BC-3F7E1ACB245E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A34CA78-5B2C-4775-B8FA-8FB981A4E34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -104,11 +103,42 @@
     <t>OFFICIELS TABLE DE MARQUE (OTM)</t>
   </si>
   <si>
+    <t>Remarques :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nom du rédacteur :  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Téléphone du rédacteur: </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A compléter et à envoyer par mail (photo) à </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri (Corps)"/>
+      </rPr>
+      <t>sportiveminicd31@gmail.com</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> en cas de non respect des entrées en jeu ou de blessure entrainant un changement de joueurs(ses).</t>
+    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
         <u/>
-        <sz val="10"/>
+        <sz val="9"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri (Corps)"/>
       </rPr>
@@ -116,9 +146,10 @@
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
+        <sz val="9"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 - opposition à 4 jrs(ses): les 4 enfants jouent 4 périodes.
@@ -127,43 +158,12 @@
 			</t>
     </r>
   </si>
-  <si>
-    <t>Remarques :</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nom du rédacteur :  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Téléphone du rédacteur: </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">A compléter et à envoyer par mail (photo) à </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri (Corps)"/>
-      </rPr>
-      <t>sportiveminicd31@gmail.com</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> en cas de non respect des entrées en jeu ou de blessure entrainant un changement de joueurs(ses).</t>
-    </r>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -250,18 +250,6 @@
       <name val="Calibri (Corps)"/>
     </font>
     <font>
-      <b/>
-      <u/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri (Corps)"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <u/>
       <sz val="9"/>
       <color rgb="FF000000"/>
@@ -271,6 +259,26 @@
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri (Corps)"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -752,69 +760,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -856,6 +801,69 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -879,15 +887,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>1</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>2</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>361950</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:colOff>106680</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>431942</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -909,8 +917,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="695325" cy="838200"/>
+          <a:off x="1" y="2"/>
+          <a:ext cx="434339" cy="431940"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -924,13 +932,13 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>962025</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:rowOff>9527</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>160020</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>733425</xdr:rowOff>
+      <xdr:rowOff>424549</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -952,8 +960,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1647825" cy="723900"/>
+          <a:off x="3773805" y="9527"/>
+          <a:ext cx="1163955" cy="415022"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1297,37 +1305,37 @@
     <col min="11" max="11" width="33" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="60.6" customHeight="1">
-      <c r="A1" s="65" t="s">
+    <row r="1" spans="1:8" ht="35.4" customHeight="1">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-    </row>
-    <row r="2" spans="1:8" ht="19.2" customHeight="1">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="66" t="s">
+      <c r="C2" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="66"/>
-      <c r="E2" s="67" t="s">
+      <c r="D2" s="45"/>
+      <c r="E2" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="68"/>
-      <c r="G2" s="69" t="s">
+      <c r="F2" s="47"/>
+      <c r="G2" s="48" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="70"/>
-    </row>
-    <row r="3" spans="1:8" ht="19.2" customHeight="1">
+      <c r="H2" s="49"/>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="4"/>
       <c r="B3" s="2" t="s">
         <v>5</v>
@@ -1336,10 +1344,10 @@
       <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="71"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="72"/>
-      <c r="H3" s="73"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="52"/>
     </row>
     <row r="4" spans="1:8" ht="7.5" customHeight="1">
       <c r="B4" s="5"/>
@@ -1351,42 +1359,42 @@
       <c r="H4" s="5"/>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
-      <c r="A5" s="62" t="s">
+      <c r="A5" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="63"/>
-      <c r="C5" s="63"/>
-      <c r="D5" s="63"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="64"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="43"/>
     </row>
     <row r="6" spans="1:8" ht="13.05" customHeight="1">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="52" t="s">
+      <c r="B6" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="52" t="s">
+      <c r="D6" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="54" t="s">
+      <c r="E6" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="55"/>
-      <c r="G6" s="55"/>
-      <c r="H6" s="56"/>
+      <c r="F6" s="56"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="57"/>
     </row>
     <row r="7" spans="1:8" ht="13.05" customHeight="1">
-      <c r="A7" s="53"/>
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="53"/>
+      <c r="A7" s="54"/>
+      <c r="B7" s="54"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="54"/>
       <c r="E7" s="7" t="s">
         <v>13</v>
       </c>
@@ -1400,7 +1408,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="19.2" customHeight="1">
+    <row r="8" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A8" s="10"/>
       <c r="B8" s="11"/>
       <c r="C8" s="12"/>
@@ -1410,7 +1418,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="18" customHeight="1">
+    <row r="9" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A9" s="10"/>
       <c r="B9" s="11"/>
       <c r="C9" s="12"/>
@@ -1420,7 +1428,7 @@
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
     </row>
-    <row r="10" spans="1:8" ht="18" customHeight="1">
+    <row r="10" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A10" s="10"/>
       <c r="B10" s="11"/>
       <c r="C10" s="12"/>
@@ -1430,7 +1438,7 @@
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1">
+    <row r="11" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A11" s="10"/>
       <c r="B11" s="11"/>
       <c r="C11" s="12"/>
@@ -1440,7 +1448,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="18" customHeight="1">
+    <row r="12" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A12" s="10"/>
       <c r="B12" s="11"/>
       <c r="C12" s="12"/>
@@ -1450,7 +1458,7 @@
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
     </row>
-    <row r="13" spans="1:8" ht="18" customHeight="1">
+    <row r="13" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A13" s="10"/>
       <c r="B13" s="11"/>
       <c r="C13" s="12"/>
@@ -1462,42 +1470,42 @@
     </row>
     <row r="14" spans="1:8" ht="10.050000000000001" customHeight="1"/>
     <row r="15" spans="1:8" ht="16.95" customHeight="1">
-      <c r="A15" s="62" t="s">
+      <c r="A15" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
-      <c r="G15" s="63"/>
-      <c r="H15" s="64"/>
+      <c r="B15" s="42"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="42"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="43"/>
     </row>
     <row r="16" spans="1:8" ht="13.05" customHeight="1">
-      <c r="A16" s="52" t="s">
+      <c r="A16" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="52" t="s">
+      <c r="B16" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="52" t="s">
+      <c r="C16" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="52" t="s">
+      <c r="D16" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="54" t="s">
+      <c r="E16" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="55"/>
-      <c r="G16" s="55"/>
-      <c r="H16" s="56"/>
+      <c r="F16" s="56"/>
+      <c r="G16" s="56"/>
+      <c r="H16" s="57"/>
     </row>
     <row r="17" spans="1:8" ht="13.05" customHeight="1">
-      <c r="A17" s="53"/>
-      <c r="B17" s="53"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
+      <c r="A17" s="54"/>
+      <c r="B17" s="54"/>
+      <c r="C17" s="54"/>
+      <c r="D17" s="54"/>
       <c r="E17" s="14" t="s">
         <v>18</v>
       </c>
@@ -1511,7 +1519,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="18" customHeight="1">
+    <row r="18" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A18" s="10"/>
       <c r="B18" s="11"/>
       <c r="C18" s="12"/>
@@ -1521,7 +1529,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1">
+    <row r="19" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A19" s="10"/>
       <c r="B19" s="11"/>
       <c r="C19" s="12"/>
@@ -1531,7 +1539,7 @@
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
     </row>
-    <row r="20" spans="1:8" ht="18" customHeight="1">
+    <row r="20" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A20" s="10"/>
       <c r="B20" s="11"/>
       <c r="C20" s="12"/>
@@ -1541,7 +1549,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="18" customHeight="1">
+    <row r="21" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A21" s="10"/>
       <c r="B21" s="11"/>
       <c r="C21" s="12"/>
@@ -1551,7 +1559,7 @@
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
     </row>
-    <row r="22" spans="1:8" ht="18" customHeight="1">
+    <row r="22" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A22" s="10"/>
       <c r="B22" s="11"/>
       <c r="C22" s="12"/>
@@ -1561,7 +1569,7 @@
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" ht="18" customHeight="1">
+    <row r="23" spans="1:8" ht="17.399999999999999" customHeight="1">
       <c r="A23" s="10"/>
       <c r="B23" s="11"/>
       <c r="C23" s="12"/>
@@ -1581,130 +1589,130 @@
       <c r="G24" s="19"/>
     </row>
     <row r="25" spans="1:8" ht="16.05" customHeight="1">
-      <c r="A25" s="41" t="s">
+      <c r="A25" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="42"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="57"/>
-      <c r="F25" s="57"/>
-      <c r="G25" s="57"/>
-      <c r="H25" s="57"/>
+      <c r="B25" s="60"/>
+      <c r="C25" s="60"/>
+      <c r="D25" s="61"/>
+      <c r="E25" s="62"/>
+      <c r="F25" s="62"/>
+      <c r="G25" s="62"/>
+      <c r="H25" s="62"/>
     </row>
     <row r="26" spans="1:8" ht="16.05" customHeight="1">
-      <c r="A26" s="58" t="s">
+      <c r="A26" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="59"/>
+      <c r="B26" s="64"/>
       <c r="C26" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D26" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E26" s="57"/>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57"/>
-    </row>
-    <row r="27" spans="1:8" ht="16.05" customHeight="1">
-      <c r="A27" s="46"/>
-      <c r="B27" s="47"/>
+      <c r="E26" s="62"/>
+      <c r="F26" s="62"/>
+      <c r="G26" s="62"/>
+      <c r="H26" s="62"/>
+    </row>
+    <row r="27" spans="1:8" ht="15" customHeight="1">
+      <c r="A27" s="65"/>
+      <c r="B27" s="66"/>
       <c r="C27" s="21"/>
       <c r="D27" s="22"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="57"/>
-      <c r="G27" s="57"/>
-      <c r="H27" s="57"/>
-    </row>
-    <row r="28" spans="1:8" ht="16.05" customHeight="1">
-      <c r="A28" s="60"/>
-      <c r="B28" s="61"/>
+      <c r="E27" s="62"/>
+      <c r="F27" s="62"/>
+      <c r="G27" s="62"/>
+      <c r="H27" s="62"/>
+    </row>
+    <row r="28" spans="1:8" ht="14.4" customHeight="1">
+      <c r="A28" s="67"/>
+      <c r="B28" s="68"/>
       <c r="C28" s="23"/>
       <c r="D28" s="24"/>
-      <c r="E28" s="57"/>
-      <c r="F28" s="57"/>
-      <c r="G28" s="57"/>
-      <c r="H28" s="57"/>
+      <c r="E28" s="62"/>
+      <c r="F28" s="62"/>
+      <c r="G28" s="62"/>
+      <c r="H28" s="62"/>
     </row>
     <row r="29" spans="1:8" ht="10.050000000000001" customHeight="1">
       <c r="A29" s="25"/>
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
-      <c r="E29" s="57"/>
-      <c r="F29" s="57"/>
-      <c r="G29" s="57"/>
-      <c r="H29" s="57"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="62"/>
+      <c r="G29" s="62"/>
+      <c r="H29" s="62"/>
     </row>
     <row r="30" spans="1:8" ht="16.05" customHeight="1">
-      <c r="A30" s="41" t="s">
+      <c r="A30" s="59" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="42"/>
-      <c r="C30" s="42"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="57"/>
-      <c r="F30" s="57"/>
-      <c r="G30" s="57"/>
-      <c r="H30" s="57"/>
+      <c r="B30" s="60"/>
+      <c r="C30" s="60"/>
+      <c r="D30" s="61"/>
+      <c r="E30" s="62"/>
+      <c r="F30" s="62"/>
+      <c r="G30" s="62"/>
+      <c r="H30" s="62"/>
     </row>
     <row r="31" spans="1:8" ht="16.05" customHeight="1">
-      <c r="A31" s="44" t="s">
+      <c r="A31" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="B31" s="45"/>
+      <c r="B31" s="70"/>
       <c r="C31" s="6" t="s">
         <v>24</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E31" s="57"/>
-      <c r="F31" s="57"/>
-      <c r="G31" s="57"/>
-      <c r="H31" s="57"/>
-    </row>
-    <row r="32" spans="1:8" s="26" customFormat="1" ht="16.05" customHeight="1">
-      <c r="A32" s="46"/>
-      <c r="B32" s="47"/>
+      <c r="E31" s="62"/>
+      <c r="F31" s="62"/>
+      <c r="G31" s="62"/>
+      <c r="H31" s="62"/>
+    </row>
+    <row r="32" spans="1:8" s="26" customFormat="1" ht="15" customHeight="1">
+      <c r="A32" s="65"/>
+      <c r="B32" s="66"/>
       <c r="C32" s="21"/>
       <c r="D32" s="22"/>
-      <c r="E32" s="57"/>
-      <c r="F32" s="57"/>
-      <c r="G32" s="57"/>
-      <c r="H32" s="57"/>
-    </row>
-    <row r="33" spans="1:8" s="26" customFormat="1" ht="16.05" customHeight="1">
-      <c r="A33" s="48"/>
-      <c r="B33" s="49"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="62"/>
+      <c r="G32" s="62"/>
+      <c r="H32" s="62"/>
+    </row>
+    <row r="33" spans="1:8" s="26" customFormat="1" ht="15" customHeight="1">
+      <c r="A33" s="71"/>
+      <c r="B33" s="72"/>
       <c r="C33" s="27"/>
       <c r="D33" s="28"/>
-      <c r="E33" s="57"/>
-      <c r="F33" s="57"/>
-      <c r="G33" s="57"/>
-      <c r="H33" s="57"/>
+      <c r="E33" s="62"/>
+      <c r="F33" s="62"/>
+      <c r="G33" s="62"/>
+      <c r="H33" s="62"/>
     </row>
     <row r="34" spans="1:8" s="26" customFormat="1" ht="4.95" customHeight="1">
       <c r="A34" s="29"/>
     </row>
-    <row r="35" spans="1:8" ht="64.05" customHeight="1">
-      <c r="A35" s="50" t="s">
-        <v>27</v>
-      </c>
-      <c r="B35" s="50"/>
-      <c r="C35" s="50"/>
-      <c r="D35" s="50"/>
-      <c r="E35" s="50"/>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="H35" s="50"/>
+    <row r="35" spans="1:8" ht="49.8" customHeight="1">
+      <c r="A35" s="73" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="73"/>
+      <c r="C35" s="73"/>
+      <c r="D35" s="73"/>
+      <c r="E35" s="73"/>
+      <c r="F35" s="73"/>
+      <c r="G35" s="73"/>
+      <c r="H35" s="73"/>
     </row>
     <row r="36" spans="1:8" ht="4.95" customHeight="1"/>
     <row r="37" spans="1:8">
       <c r="A37" s="30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B37" s="31"/>
       <c r="C37" s="31"/>
@@ -1714,7 +1722,7 @@
       <c r="G37" s="31"/>
       <c r="H37" s="32"/>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" ht="12.6" customHeight="1">
       <c r="A38" s="33"/>
       <c r="H38" s="34"/>
     </row>
@@ -1726,7 +1734,7 @@
       <c r="A40" s="33"/>
       <c r="H40" s="34"/>
     </row>
-    <row r="41" spans="1:8" ht="24" customHeight="1">
+    <row r="41" spans="1:8" ht="15.6" customHeight="1">
       <c r="A41" s="33"/>
       <c r="H41" s="34"/>
     </row>
@@ -1734,18 +1742,18 @@
       <c r="A42" s="33"/>
       <c r="H42" s="34"/>
     </row>
-    <row r="43" spans="1:8" ht="15" customHeight="1">
+    <row r="43" spans="1:8" ht="13.8" customHeight="1">
       <c r="A43" s="33"/>
       <c r="H43" s="34"/>
     </row>
     <row r="44" spans="1:8" ht="15" customHeight="1">
       <c r="A44" s="35" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B44" s="36"/>
       <c r="C44" s="37"/>
       <c r="D44" s="38" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E44" s="39"/>
       <c r="F44" s="39"/>
@@ -1753,41 +1761,29 @@
       <c r="H44" s="40"/>
     </row>
     <row r="45" spans="1:8">
-      <c r="A45" s="51" t="s">
-        <v>31</v>
-      </c>
-      <c r="B45" s="51"/>
-      <c r="C45" s="51"/>
-      <c r="D45" s="51"/>
-      <c r="E45" s="51"/>
-      <c r="F45" s="51"/>
-      <c r="G45" s="51"/>
-      <c r="H45" s="51"/>
+      <c r="A45" s="58" t="s">
+        <v>30</v>
+      </c>
+      <c r="B45" s="58"/>
+      <c r="C45" s="58"/>
+      <c r="D45" s="58"/>
+      <c r="E45" s="58"/>
+      <c r="F45" s="58"/>
+      <c r="G45" s="58"/>
+      <c r="H45" s="58"/>
     </row>
     <row r="46" spans="1:8">
-      <c r="A46" s="51"/>
-      <c r="B46" s="51"/>
-      <c r="C46" s="51"/>
-      <c r="D46" s="51"/>
-      <c r="E46" s="51"/>
-      <c r="F46" s="51"/>
-      <c r="G46" s="51"/>
-      <c r="H46" s="51"/>
+      <c r="A46" s="58"/>
+      <c r="B46" s="58"/>
+      <c r="C46" s="58"/>
+      <c r="D46" s="58"/>
+      <c r="E46" s="58"/>
+      <c r="F46" s="58"/>
+      <c r="G46" s="58"/>
+      <c r="H46" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:H6"/>
     <mergeCell ref="A45:H46"/>
     <mergeCell ref="A16:A17"/>
     <mergeCell ref="B16:B17"/>
@@ -1804,6 +1800,18 @@
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:H6"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B24" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -1811,6 +1819,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>